<commit_message>
10+ more question solved
</commit_message>
<xml_diff>
--- a/array.xlsx
+++ b/array.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soumyajit\Downloads\07-03-2026\Coding_Practice\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE8EC21-25D9-4EC7-9968-9EA55317D1FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="60" windowWidth="20115" windowHeight="8010"/>
+    <workbookView xWindow="3000" yWindow="3000" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -16,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="27">
   <si>
     <t>Find the smallest number in an array</t>
   </si>
@@ -102,7 +108,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -144,14 +150,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -189,7 +198,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -261,7 +270,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -434,14 +443,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="55.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="55.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -449,7 +458,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -457,7 +466,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -465,7 +474,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -473,109 +482,172 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -585,18 +657,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>